<commit_message>
Done till page 23
</commit_message>
<xml_diff>
--- a/Report_format/BSLABP26-27.xlsx
+++ b/Report_format/BSLABP26-27.xlsx
@@ -13,19 +13,16 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PLAN SUMMARY'!$A$1:$N$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PLAN SUMMARY'!$A$2:$R$27</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
   <si>
     <t>APP / BSL</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> PLAN SUMMARY 2026-27</t>
   </si>
   <si>
     <t>UNIT : '000 T</t>
@@ -159,6 +156,18 @@
   <si>
     <t>( 1 )</t>
   </si>
+  <si>
+    <t>HR Coil</t>
+  </si>
+  <si>
+    <t>HR Plate</t>
+  </si>
+  <si>
+    <t>HR Sheet</t>
+  </si>
+  <si>
+    <t>BSL  PLAN SUMMARY 2026-27</t>
+  </si>
 </sst>
 </file>
 
@@ -169,7 +178,7 @@
     <numFmt numFmtId="165" formatCode="0_)"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -245,27 +254,8 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FF002060"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -275,13 +265,6 @@
       <color rgb="FF002060"/>
       <name val="Courier"/>
       <family val="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -545,12 +528,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -559,9 +541,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -570,96 +549,15 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -681,43 +579,25 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="11" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -726,7 +606,7 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -756,43 +636,22 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="11" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -815,6 +674,19 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
@@ -824,18 +696,85 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal_APP-1" xfId="1"/>
-    <cellStyle name="Normal_APP-5" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1691,6 +1630,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:X47"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
@@ -1710,18 +1652,18 @@
     <col min="14" max="14" width="7" style="1" customWidth="1"/>
     <col min="15" max="15" width="9.85546875" style="1" customWidth="1"/>
     <col min="16" max="16" width="10.5703125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="23" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="12.75" x14ac:dyDescent="0.2">
       <c r="N1" s="2"/>
     </row>
-    <row r="2" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" ht="16.5" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1730,1646 +1672,1677 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:24" ht="19.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
+      <c r="M3" s="76"/>
+      <c r="N3" s="76"/>
+    </row>
+    <row r="4" spans="1:24" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+    </row>
+    <row r="5" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-    </row>
-    <row r="4" spans="1:24" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-    </row>
-    <row r="5" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:24" s="10" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="77" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:24" s="20" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11" t="s">
+      <c r="C6" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="D6" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="E6" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="F6" s="81"/>
+      <c r="G6" s="82"/>
+      <c r="H6" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16" t="s">
+      <c r="I6" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="J6" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="17" t="s">
+      <c r="K6" s="85"/>
+      <c r="L6" s="86"/>
+      <c r="M6" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="18"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="16" t="s">
+      <c r="N6" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="N6" s="16" t="s">
+      <c r="O6" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="O6" s="20" t="s">
+      <c r="P6" s="74" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="74" t="s">
+        <v>42</v>
+      </c>
+      <c r="R6" s="74" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" s="10" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:24" s="20" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="21" t="s">
+      <c r="B7" s="78"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="78"/>
+      <c r="E7" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="12" t="s">
+      <c r="F7" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="G7" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="H7" s="83"/>
+      <c r="I7" s="83"/>
+      <c r="J7" s="87"/>
+      <c r="K7" s="88"/>
+      <c r="L7" s="89"/>
+      <c r="M7" s="83"/>
+      <c r="N7" s="83"/>
+      <c r="O7" s="83"/>
+      <c r="P7" s="83"/>
+      <c r="Q7" s="83"/>
+      <c r="R7" s="83"/>
+    </row>
+    <row r="8" spans="1:24" s="10" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="11"/>
+      <c r="B8" s="78"/>
+      <c r="C8" s="69"/>
+      <c r="D8" s="78"/>
+      <c r="E8" s="69"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="83"/>
+      <c r="I8" s="83"/>
+      <c r="J8" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="28"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-    </row>
-    <row r="8" spans="1:24" s="20" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="21"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="16" t="s">
+      <c r="K8" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="16" t="s">
+      <c r="L8" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="L8" s="16" t="s">
+      <c r="M8" s="83"/>
+      <c r="N8" s="83"/>
+      <c r="O8" s="83"/>
+      <c r="P8" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="25"/>
-      <c r="N8" s="25"/>
-      <c r="P8" s="30" t="s">
+      <c r="Q8" s="83" t="s">
+        <v>19</v>
+      </c>
+      <c r="R8" s="83" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" s="10" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="12"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="70"/>
+      <c r="D9" s="79"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="73"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="75"/>
+      <c r="I9" s="75"/>
+      <c r="J9" s="75"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="75"/>
+      <c r="M9" s="75"/>
+      <c r="N9" s="75"/>
+      <c r="O9" s="75"/>
+      <c r="P9" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="R8" s="32" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" s="20" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="33"/>
-      <c r="B9" s="34"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="37"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="P9" s="38" t="s">
+      <c r="Q9" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="Q9" s="39" t="s">
+      <c r="R9" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="R9" s="40" t="s">
+    </row>
+    <row r="10" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="42">
+      <c r="B10" s="14">
         <f>+'[1]S-2'!B9</f>
         <v>525</v>
       </c>
-      <c r="C10" s="43">
+      <c r="C10" s="15">
         <f>'[1]S-2'!D9</f>
         <v>513</v>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="16">
         <f>'[1]S-2'!F9</f>
         <v>461</v>
       </c>
-      <c r="E10" s="43">
+      <c r="E10" s="15">
         <f>+G10+F10</f>
         <v>443</v>
       </c>
-      <c r="F10" s="45">
+      <c r="F10" s="17">
         <f>+'[1]S-3'!C10</f>
         <v>106</v>
       </c>
-      <c r="G10" s="45">
+      <c r="G10" s="17">
         <f>+'[1]S-3'!D10</f>
         <v>337</v>
       </c>
-      <c r="H10" s="45">
+      <c r="H10" s="17">
         <f>'[1]S-4'!B9</f>
         <v>356</v>
       </c>
-      <c r="I10" s="44">
+      <c r="I10" s="16">
         <f>'[1]S-4'!L9</f>
         <v>38</v>
       </c>
-      <c r="J10" s="43">
+      <c r="J10" s="15">
         <f>+'[1]S-9'!I8</f>
         <v>55</v>
       </c>
-      <c r="K10" s="46">
+      <c r="K10" s="18">
         <f>+'[1]S-9'!M8</f>
         <v>83.5</v>
       </c>
-      <c r="L10" s="46">
+      <c r="L10" s="18">
         <f>+J10+K10</f>
         <v>138.5</v>
       </c>
-      <c r="M10" s="46">
+      <c r="M10" s="18">
         <f>'[1]S-9'!N8</f>
         <v>388</v>
       </c>
-      <c r="N10" s="47">
+      <c r="N10" s="19">
         <f>'[1]S-2'!I9</f>
         <v>0.5</v>
       </c>
-      <c r="O10" s="48">
+      <c r="O10" s="19">
         <v>45</v>
       </c>
-      <c r="P10" s="49">
+      <c r="P10" s="19">
         <v>166.5</v>
       </c>
-      <c r="Q10" s="50">
+      <c r="Q10" s="19">
         <v>35</v>
       </c>
-      <c r="R10" s="51">
+      <c r="R10" s="19">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="52">
+    <row r="11" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="20">
         <f>+'[1]S-2'!B10</f>
         <v>565</v>
       </c>
-      <c r="C11" s="47">
+      <c r="C11" s="19">
         <f>'[1]S-2'!D10</f>
         <v>587</v>
       </c>
-      <c r="D11" s="44">
+      <c r="D11" s="16">
         <f>'[1]S-2'!F10</f>
         <v>475</v>
       </c>
-      <c r="E11" s="47">
+      <c r="E11" s="19">
         <f>+G11+F11</f>
         <v>454</v>
       </c>
-      <c r="F11" s="46">
+      <c r="F11" s="18">
         <f>+'[1]S-3'!C11</f>
         <v>109</v>
       </c>
-      <c r="G11" s="46">
+      <c r="G11" s="18">
         <f>+'[1]S-3'!D11</f>
         <v>345</v>
       </c>
-      <c r="H11" s="46">
+      <c r="H11" s="18">
         <f>'[1]S-4'!B10</f>
         <v>315</v>
       </c>
-      <c r="I11" s="44">
+      <c r="I11" s="16">
         <f>'[1]S-4'!L10</f>
         <v>51</v>
       </c>
-      <c r="J11" s="47">
+      <c r="J11" s="19">
         <f>+'[1]S-9'!I9</f>
         <v>57</v>
       </c>
-      <c r="K11" s="46">
+      <c r="K11" s="18">
         <f>+'[1]S-9'!M9</f>
         <v>86.5</v>
       </c>
-      <c r="L11" s="46">
+      <c r="L11" s="18">
         <f>+J11+K11</f>
         <v>143.5</v>
       </c>
-      <c r="M11" s="46">
+      <c r="M11" s="18">
         <f>'[1]S-9'!N9</f>
         <v>351</v>
       </c>
-      <c r="N11" s="47">
+      <c r="N11" s="19">
         <f>'[1]S-2'!I10</f>
         <v>2.69</v>
       </c>
-      <c r="O11" s="48">
+      <c r="O11" s="19">
         <v>50</v>
       </c>
-      <c r="P11" s="49">
+      <c r="P11" s="19">
         <v>106.5</v>
       </c>
-      <c r="Q11" s="50">
+      <c r="Q11" s="19">
         <v>39</v>
       </c>
-      <c r="R11" s="49">
+      <c r="R11" s="19">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="52">
+    <row r="12" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="20">
         <f>+'[1]S-2'!B11</f>
         <v>547</v>
       </c>
-      <c r="C12" s="47">
+      <c r="C12" s="19">
         <f>'[1]S-2'!D11</f>
         <v>537</v>
       </c>
-      <c r="D12" s="44">
+      <c r="D12" s="16">
         <f>'[1]S-2'!F11</f>
         <v>469</v>
       </c>
-      <c r="E12" s="53">
+      <c r="E12" s="21">
         <f>+G12+F12</f>
         <v>451</v>
       </c>
-      <c r="F12" s="46">
+      <c r="F12" s="18">
         <f>+'[1]S-3'!C12</f>
         <v>121</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="18">
         <f>+'[1]S-3'!D12</f>
         <v>330</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="18">
         <f>'[1]S-4'!B11</f>
         <v>380</v>
       </c>
-      <c r="I12" s="44">
+      <c r="I12" s="16">
         <f>'[1]S-4'!L11</f>
         <v>51.5</v>
       </c>
-      <c r="J12" s="47">
+      <c r="J12" s="19">
         <f>+'[1]S-9'!I10</f>
         <v>45.000000000000007</v>
       </c>
-      <c r="K12" s="46">
+      <c r="K12" s="18">
         <f>+'[1]S-9'!M10</f>
         <v>83.5</v>
       </c>
-      <c r="L12" s="46">
+      <c r="L12" s="18">
         <f>+J12+K12</f>
         <v>128.5</v>
       </c>
-      <c r="M12" s="46">
+      <c r="M12" s="18">
         <f>'[1]S-9'!N10</f>
         <v>413</v>
       </c>
-      <c r="N12" s="47">
+      <c r="N12" s="19">
         <f>'[1]S-2'!I11</f>
         <v>0</v>
       </c>
-      <c r="O12" s="48">
+      <c r="O12" s="19">
         <v>45.5</v>
       </c>
-      <c r="P12" s="49">
+      <c r="P12" s="19">
         <v>187.5</v>
       </c>
-      <c r="Q12" s="50">
+      <c r="Q12" s="19">
         <v>39</v>
       </c>
-      <c r="R12" s="54">
+      <c r="R12" s="19">
         <v>12.5</v>
       </c>
     </row>
-    <row r="13" spans="1:24" s="63" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="55" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="56">
+    <row r="13" spans="1:24" s="29" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="23">
         <f>(B10*30+B11*31+B12*30)/91</f>
         <v>545.87912087912093</v>
       </c>
-      <c r="C13" s="57">
+      <c r="C13" s="24">
         <f>SUM(C10:C12)</f>
         <v>1637</v>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="24">
         <f t="shared" ref="D13:N13" si="0">SUM(D10:D12)</f>
         <v>1405</v>
       </c>
-      <c r="E13" s="57">
+      <c r="E13" s="24">
         <f t="shared" si="0"/>
         <v>1348</v>
       </c>
-      <c r="F13" s="57">
+      <c r="F13" s="24">
         <f>SUM(F10:F12)</f>
         <v>336</v>
       </c>
-      <c r="G13" s="57">
+      <c r="G13" s="24">
         <f t="shared" si="0"/>
         <v>1012</v>
       </c>
-      <c r="H13" s="57">
+      <c r="H13" s="24">
         <f t="shared" si="0"/>
         <v>1051</v>
       </c>
-      <c r="I13" s="58">
+      <c r="I13" s="25">
         <f t="shared" si="0"/>
         <v>140.5</v>
       </c>
-      <c r="J13" s="58">
+      <c r="J13" s="25">
         <f t="shared" si="0"/>
         <v>157</v>
       </c>
-      <c r="K13" s="58">
+      <c r="K13" s="25">
         <f t="shared" si="0"/>
         <v>253.5</v>
       </c>
-      <c r="L13" s="58">
+      <c r="L13" s="25">
         <f t="shared" si="0"/>
         <v>410.5</v>
       </c>
-      <c r="M13" s="56">
+      <c r="M13" s="23">
         <f t="shared" si="0"/>
         <v>1152</v>
       </c>
-      <c r="N13" s="59">
+      <c r="N13" s="26">
         <f t="shared" si="0"/>
         <v>3.19</v>
       </c>
-      <c r="O13" s="48">
+      <c r="O13" s="26">
         <v>140.5</v>
       </c>
-      <c r="P13" s="60">
+      <c r="P13" s="26">
         <v>460.5</v>
       </c>
-      <c r="Q13" s="60">
+      <c r="Q13" s="26">
         <v>113</v>
       </c>
-      <c r="R13" s="60">
+      <c r="R13" s="26">
         <v>27.5</v>
       </c>
-      <c r="S13" s="61"/>
-      <c r="T13" s="61"/>
-      <c r="U13" s="61"/>
-      <c r="V13" s="61"/>
-      <c r="W13" s="61"/>
-      <c r="X13" s="62"/>
-    </row>
-    <row r="14" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="64" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="42">
+      <c r="S13" s="27"/>
+      <c r="T13" s="27"/>
+      <c r="U13" s="27"/>
+      <c r="V13" s="27"/>
+      <c r="W13" s="27"/>
+      <c r="X13" s="28"/>
+    </row>
+    <row r="14" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="14">
         <f>+'[1]S-2'!B13</f>
         <v>506</v>
       </c>
-      <c r="C14" s="65">
+      <c r="C14" s="31">
         <f>'[1]S-2'!D13</f>
         <v>528</v>
       </c>
-      <c r="D14" s="44">
+      <c r="D14" s="16">
         <f>'[1]S-2'!F13</f>
         <v>448</v>
       </c>
-      <c r="E14" s="43">
+      <c r="E14" s="15">
         <f>+G14+F14</f>
         <v>425</v>
       </c>
-      <c r="F14" s="45">
+      <c r="F14" s="17">
         <f>+'[1]S-3'!C14</f>
         <v>121</v>
       </c>
-      <c r="G14" s="45">
+      <c r="G14" s="17">
         <f>+'[1]S-3'!D14</f>
         <v>304</v>
       </c>
-      <c r="H14" s="47">
+      <c r="H14" s="19">
         <f>'[1]S-4'!B13</f>
         <v>395</v>
       </c>
-      <c r="I14" s="66">
+      <c r="I14" s="32">
         <f>'[1]S-4'!L13</f>
         <v>52.5</v>
       </c>
-      <c r="J14" s="67">
+      <c r="J14" s="33">
         <f>+'[1]S-9'!I12</f>
         <v>57</v>
       </c>
-      <c r="K14" s="68">
+      <c r="K14" s="34">
         <f>+'[1]S-9'!M12</f>
         <v>86</v>
       </c>
-      <c r="L14" s="68">
+      <c r="L14" s="34">
         <f>+J14+K14</f>
         <v>143</v>
       </c>
-      <c r="M14" s="46">
+      <c r="M14" s="18">
         <f>'[1]S-9'!N12</f>
         <v>423</v>
       </c>
-      <c r="N14" s="69">
+      <c r="N14" s="35">
         <f>'[1]S-2'!I13</f>
         <v>4.95</v>
       </c>
-      <c r="O14" s="48">
+      <c r="O14" s="35">
         <v>42</v>
       </c>
-      <c r="P14" s="49">
+      <c r="P14" s="35">
         <v>185</v>
       </c>
-      <c r="Q14" s="50">
+      <c r="Q14" s="35">
         <v>39</v>
       </c>
-      <c r="R14" s="51">
+      <c r="R14" s="35">
         <v>13.5</v>
       </c>
     </row>
-    <row r="15" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="64" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="52">
+    <row r="15" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="20">
         <f>+'[1]S-2'!B14</f>
         <v>507</v>
       </c>
-      <c r="C15" s="70">
+      <c r="C15" s="36">
         <f>'[1]S-2'!D14</f>
         <v>493</v>
       </c>
-      <c r="D15" s="44">
+      <c r="D15" s="16">
         <f>'[1]S-2'!F14</f>
         <v>438</v>
       </c>
-      <c r="E15" s="47">
+      <c r="E15" s="19">
         <f>+G15+F15</f>
         <v>416</v>
       </c>
-      <c r="F15" s="46">
+      <c r="F15" s="18">
         <f>+'[1]S-3'!C15</f>
         <v>77</v>
       </c>
-      <c r="G15" s="46">
+      <c r="G15" s="18">
         <f>+'[1]S-3'!D15</f>
         <v>339</v>
       </c>
-      <c r="H15" s="47">
+      <c r="H15" s="19">
         <f>'[1]S-4'!B14</f>
         <v>405</v>
       </c>
-      <c r="I15" s="66">
+      <c r="I15" s="32">
         <f>'[1]S-4'!L14</f>
         <v>52.5</v>
       </c>
-      <c r="J15" s="71">
+      <c r="J15" s="37">
         <f>+'[1]S-9'!I13</f>
         <v>57</v>
       </c>
-      <c r="K15" s="68">
+      <c r="K15" s="34">
         <f>+'[1]S-9'!M13</f>
         <v>86</v>
       </c>
-      <c r="L15" s="68">
+      <c r="L15" s="34">
         <f>+J15+K15</f>
         <v>143</v>
       </c>
-      <c r="M15" s="46">
+      <c r="M15" s="18">
         <f>'[1]S-9'!N13</f>
         <v>432</v>
       </c>
-      <c r="N15" s="69">
+      <c r="N15" s="35">
         <f>'[1]S-2'!I14</f>
         <v>5.21</v>
       </c>
-      <c r="O15" s="48">
+      <c r="O15" s="35">
         <v>41</v>
       </c>
-      <c r="P15" s="49">
+      <c r="P15" s="35">
         <v>195</v>
       </c>
-      <c r="Q15" s="50">
+      <c r="Q15" s="35">
         <v>39</v>
       </c>
-      <c r="R15" s="49">
+      <c r="R15" s="35">
         <v>13.5</v>
       </c>
     </row>
-    <row r="16" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="64" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="52">
+    <row r="16" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="20">
         <f>+'[1]S-2'!B15</f>
         <v>507</v>
       </c>
-      <c r="C16" s="72">
+      <c r="C16" s="38">
         <f>'[1]S-2'!D15</f>
         <v>515</v>
       </c>
-      <c r="D16" s="53">
+      <c r="D16" s="21">
         <f>'[1]S-2'!F15</f>
         <v>465</v>
       </c>
-      <c r="E16" s="53">
+      <c r="E16" s="21">
         <f>+G16+F16</f>
         <v>447</v>
       </c>
-      <c r="F16" s="46">
+      <c r="F16" s="18">
         <f>+'[1]S-3'!C16</f>
         <v>113</v>
       </c>
-      <c r="G16" s="46">
+      <c r="G16" s="18">
         <f>+'[1]S-3'!D16</f>
         <v>334</v>
       </c>
-      <c r="H16" s="47">
+      <c r="H16" s="19">
         <f>'[1]S-4'!B15</f>
         <v>390</v>
       </c>
-      <c r="I16" s="66">
+      <c r="I16" s="32">
         <f>'[1]S-4'!L15</f>
         <v>51</v>
       </c>
-      <c r="J16" s="71">
+      <c r="J16" s="37">
         <f>+'[1]S-9'!I14</f>
         <v>55</v>
       </c>
-      <c r="K16" s="68">
+      <c r="K16" s="34">
         <f>+'[1]S-9'!M14</f>
         <v>83.5</v>
       </c>
-      <c r="L16" s="68">
+      <c r="L16" s="34">
         <f>+J16+K16</f>
         <v>138.5</v>
       </c>
-      <c r="M16" s="46">
+      <c r="M16" s="18">
         <f>'[1]S-9'!N14</f>
         <v>416</v>
       </c>
-      <c r="N16" s="69">
+      <c r="N16" s="35">
         <f>'[1]S-2'!I15</f>
         <v>0.25</v>
       </c>
-      <c r="O16" s="48">
+      <c r="O16" s="35">
         <v>39.5</v>
       </c>
-      <c r="P16" s="49">
+      <c r="P16" s="35">
         <v>187</v>
       </c>
-      <c r="Q16" s="50">
+      <c r="Q16" s="35">
         <v>39</v>
       </c>
-      <c r="R16" s="54">
+      <c r="R16" s="35">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:24" s="63" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="55" t="s">
-        <v>31</v>
-      </c>
-      <c r="B17" s="73">
+    <row r="17" spans="1:24" s="29" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="39">
         <f>(B14*31+B15*31+B16*30)/92</f>
         <v>506.66304347826087</v>
       </c>
-      <c r="C17" s="57">
+      <c r="C17" s="24">
         <f t="shared" ref="C17:N17" si="1">SUM(C14:C16)</f>
         <v>1536</v>
       </c>
-      <c r="D17" s="57">
+      <c r="D17" s="24">
         <f t="shared" si="1"/>
         <v>1351</v>
       </c>
-      <c r="E17" s="57">
+      <c r="E17" s="24">
         <f t="shared" si="1"/>
         <v>1288</v>
       </c>
-      <c r="F17" s="57">
+      <c r="F17" s="24">
         <f>SUM(F14:F16)</f>
         <v>311</v>
       </c>
-      <c r="G17" s="57">
+      <c r="G17" s="24">
         <f t="shared" si="1"/>
         <v>977</v>
       </c>
-      <c r="H17" s="57">
+      <c r="H17" s="24">
         <f t="shared" si="1"/>
         <v>1190</v>
       </c>
-      <c r="I17" s="58">
+      <c r="I17" s="25">
         <f t="shared" si="1"/>
         <v>156</v>
       </c>
-      <c r="J17" s="58">
+      <c r="J17" s="25">
         <f t="shared" si="1"/>
         <v>169</v>
       </c>
-      <c r="K17" s="58">
+      <c r="K17" s="25">
         <f t="shared" si="1"/>
         <v>255.5</v>
       </c>
-      <c r="L17" s="58">
+      <c r="L17" s="25">
         <f t="shared" si="1"/>
         <v>424.5</v>
       </c>
-      <c r="M17" s="56">
+      <c r="M17" s="23">
         <f t="shared" si="1"/>
         <v>1271</v>
       </c>
-      <c r="N17" s="59">
+      <c r="N17" s="26">
         <f t="shared" si="1"/>
         <v>10.41</v>
       </c>
-      <c r="O17" s="48">
+      <c r="O17" s="26">
         <v>122.5</v>
       </c>
-      <c r="P17" s="60">
+      <c r="P17" s="26">
         <v>567</v>
       </c>
-      <c r="Q17" s="60">
+      <c r="Q17" s="26">
         <v>117</v>
       </c>
-      <c r="R17" s="60">
+      <c r="R17" s="26">
         <v>39</v>
       </c>
-      <c r="S17" s="61"/>
-      <c r="T17" s="61"/>
-      <c r="U17" s="61"/>
-      <c r="V17" s="61"/>
-      <c r="W17" s="61"/>
-      <c r="X17" s="62"/>
-    </row>
-    <row r="18" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="64" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="42">
+      <c r="S17" s="27"/>
+      <c r="T17" s="27"/>
+      <c r="U17" s="27"/>
+      <c r="V17" s="27"/>
+      <c r="W17" s="27"/>
+      <c r="X17" s="28"/>
+    </row>
+    <row r="18" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="14">
         <f>+'[1]S-2'!B17</f>
         <v>513</v>
       </c>
-      <c r="C18" s="65">
+      <c r="C18" s="31">
         <f>'[1]S-2'!D17</f>
         <v>557</v>
       </c>
-      <c r="D18" s="44">
+      <c r="D18" s="16">
         <f>'[1]S-2'!F17</f>
         <v>437</v>
       </c>
-      <c r="E18" s="43">
+      <c r="E18" s="15">
         <f>+G18+F18</f>
         <v>413</v>
       </c>
-      <c r="F18" s="45">
+      <c r="F18" s="17">
         <f>+'[1]S-3'!C18</f>
         <v>125</v>
       </c>
-      <c r="G18" s="45">
+      <c r="G18" s="17">
         <f>+'[1]S-3'!D18</f>
         <v>288</v>
       </c>
-      <c r="H18" s="47">
+      <c r="H18" s="19">
         <f>'[1]S-4'!B17</f>
         <v>395</v>
       </c>
-      <c r="I18" s="66">
+      <c r="I18" s="32">
         <f>'[1]S-4'!L17</f>
         <v>53</v>
       </c>
-      <c r="J18" s="67">
+      <c r="J18" s="33">
         <f>+'[1]S-9'!I16</f>
         <v>57</v>
       </c>
-      <c r="K18" s="68">
+      <c r="K18" s="34">
         <f>+'[1]S-9'!M16</f>
         <v>86.5</v>
       </c>
-      <c r="L18" s="68">
+      <c r="L18" s="34">
         <f>+J18+K18</f>
         <v>143.5</v>
       </c>
-      <c r="M18" s="46">
+      <c r="M18" s="18">
         <f>'[1]S-9'!N16</f>
         <v>423</v>
       </c>
-      <c r="N18" s="69">
+      <c r="N18" s="35">
         <f>'[1]S-2'!I17</f>
         <v>6.05</v>
       </c>
-      <c r="O18" s="61">
+      <c r="O18" s="35">
         <v>42</v>
       </c>
-      <c r="P18" s="49">
+      <c r="P18" s="35">
         <v>184.5</v>
       </c>
-      <c r="Q18" s="50">
+      <c r="Q18" s="35">
         <v>40</v>
       </c>
-      <c r="R18" s="51">
+      <c r="R18" s="35">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="64" t="s">
-        <v>33</v>
-      </c>
-      <c r="B19" s="52">
+    <row r="19" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="20">
         <f>+'[1]S-2'!B18</f>
         <v>526</v>
       </c>
-      <c r="C19" s="70">
+      <c r="C19" s="36">
         <f>'[1]S-2'!D18</f>
         <v>513</v>
       </c>
-      <c r="D19" s="44">
+      <c r="D19" s="16">
         <f>'[1]S-2'!F18</f>
         <v>425</v>
       </c>
-      <c r="E19" s="47">
+      <c r="E19" s="19">
         <f>+G19+F19</f>
         <v>399</v>
       </c>
-      <c r="F19" s="46">
+      <c r="F19" s="18">
         <f>+'[1]S-3'!C19</f>
         <v>120</v>
       </c>
-      <c r="G19" s="46">
+      <c r="G19" s="18">
         <f>+'[1]S-3'!D19</f>
         <v>279</v>
       </c>
-      <c r="H19" s="47">
+      <c r="H19" s="19">
         <f>'[1]S-4'!B18</f>
         <v>380</v>
       </c>
-      <c r="I19" s="66">
+      <c r="I19" s="32">
         <f>'[1]S-4'!L18</f>
         <v>51</v>
       </c>
-      <c r="J19" s="71">
+      <c r="J19" s="37">
         <f>+'[1]S-9'!I17</f>
         <v>55.000000000000007</v>
       </c>
-      <c r="K19" s="68">
+      <c r="K19" s="34">
         <f>+'[1]S-9'!M17</f>
         <v>83.5</v>
       </c>
-      <c r="L19" s="68">
+      <c r="L19" s="34">
         <f>+J19+K19</f>
         <v>138.5</v>
       </c>
-      <c r="M19" s="46">
+      <c r="M19" s="18">
         <f>'[1]S-9'!N17</f>
         <v>407</v>
       </c>
-      <c r="N19" s="69">
+      <c r="N19" s="35">
         <f>'[1]S-2'!I18</f>
         <v>8.23</v>
       </c>
-      <c r="O19" s="48">
+      <c r="O19" s="35">
         <v>40.5</v>
       </c>
-      <c r="P19" s="49">
+      <c r="P19" s="35">
         <v>177</v>
       </c>
-      <c r="Q19" s="50">
+      <c r="Q19" s="35">
         <v>39</v>
       </c>
-      <c r="R19" s="49">
+      <c r="R19" s="35">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="64" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" s="52">
+    <row r="20" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="20">
         <f>+'[1]S-2'!B19</f>
         <v>526</v>
       </c>
-      <c r="C20" s="72">
+      <c r="C20" s="38">
         <f>'[1]S-2'!D19</f>
         <v>587</v>
       </c>
-      <c r="D20" s="53">
+      <c r="D20" s="21">
         <f>'[1]S-2'!F19</f>
         <v>478</v>
       </c>
-      <c r="E20" s="53">
+      <c r="E20" s="21">
         <f>+G20+F20</f>
         <v>459</v>
       </c>
-      <c r="F20" s="46">
+      <c r="F20" s="18">
         <f>+'[1]S-3'!C20</f>
         <v>113</v>
       </c>
-      <c r="G20" s="46">
+      <c r="G20" s="18">
         <f>+'[1]S-3'!D20</f>
         <v>346</v>
       </c>
-      <c r="H20" s="47">
+      <c r="H20" s="19">
         <f>'[1]S-4'!B19</f>
         <v>395</v>
       </c>
-      <c r="I20" s="66">
+      <c r="I20" s="32">
         <f>'[1]S-4'!L19</f>
         <v>53.5</v>
       </c>
-      <c r="J20" s="71">
+      <c r="J20" s="37">
         <f>+'[1]S-9'!I18</f>
         <v>57</v>
       </c>
-      <c r="K20" s="68">
+      <c r="K20" s="34">
         <f>+'[1]S-9'!M18</f>
         <v>70.5</v>
       </c>
-      <c r="L20" s="68">
+      <c r="L20" s="34">
         <f>+J20+K20</f>
         <v>127.5</v>
       </c>
-      <c r="M20" s="46">
+      <c r="M20" s="18">
         <f>'[1]S-9'!N18</f>
         <v>423</v>
       </c>
-      <c r="N20" s="69">
+      <c r="N20" s="35">
         <f>'[1]S-2'!I19</f>
         <v>0.76</v>
       </c>
-      <c r="O20" s="48">
+      <c r="O20" s="35">
         <v>41</v>
       </c>
-      <c r="P20" s="49">
+      <c r="P20" s="35">
         <v>201</v>
       </c>
-      <c r="Q20" s="50">
+      <c r="Q20" s="35">
         <v>40</v>
       </c>
-      <c r="R20" s="54">
+      <c r="R20" s="35">
         <v>13.5</v>
       </c>
     </row>
-    <row r="21" spans="1:24" s="63" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="55" t="s">
-        <v>35</v>
-      </c>
-      <c r="B21" s="73">
+    <row r="21" spans="1:24" s="29" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="39">
         <f>(B18*31+B19*30+B20*31)/92</f>
         <v>521.61956521739125</v>
       </c>
-      <c r="C21" s="57">
+      <c r="C21" s="24">
         <f t="shared" ref="C21:N21" si="2">SUM(C18:C20)</f>
         <v>1657</v>
       </c>
-      <c r="D21" s="57">
+      <c r="D21" s="24">
         <f t="shared" si="2"/>
         <v>1340</v>
       </c>
-      <c r="E21" s="57">
+      <c r="E21" s="24">
         <f t="shared" si="2"/>
         <v>1271</v>
       </c>
-      <c r="F21" s="57">
+      <c r="F21" s="24">
         <f>SUM(F18:F20)</f>
         <v>358</v>
       </c>
-      <c r="G21" s="57">
+      <c r="G21" s="24">
         <f t="shared" si="2"/>
         <v>913</v>
       </c>
-      <c r="H21" s="57">
+      <c r="H21" s="24">
         <f t="shared" si="2"/>
         <v>1170</v>
       </c>
-      <c r="I21" s="58">
+      <c r="I21" s="25">
         <f t="shared" si="2"/>
         <v>157.5</v>
       </c>
-      <c r="J21" s="58">
+      <c r="J21" s="25">
         <f t="shared" si="2"/>
         <v>169</v>
       </c>
-      <c r="K21" s="58">
+      <c r="K21" s="25">
         <f t="shared" si="2"/>
         <v>240.5</v>
       </c>
-      <c r="L21" s="58">
+      <c r="L21" s="25">
         <f t="shared" si="2"/>
         <v>409.5</v>
       </c>
-      <c r="M21" s="56">
+      <c r="M21" s="23">
         <f t="shared" si="2"/>
         <v>1253</v>
       </c>
-      <c r="N21" s="59">
+      <c r="N21" s="26">
         <f t="shared" si="2"/>
         <v>15.040000000000001</v>
       </c>
-      <c r="O21" s="48">
+      <c r="O21" s="26">
         <v>123.5</v>
       </c>
-      <c r="P21" s="60">
+      <c r="P21" s="26">
         <v>562.5</v>
       </c>
-      <c r="Q21" s="60">
+      <c r="Q21" s="26">
         <v>119</v>
       </c>
-      <c r="R21" s="60">
+      <c r="R21" s="26">
         <v>38.5</v>
       </c>
-      <c r="S21" s="61"/>
-      <c r="T21" s="61"/>
-      <c r="U21" s="61"/>
-      <c r="V21" s="61"/>
-      <c r="W21" s="61"/>
-      <c r="X21" s="62"/>
-    </row>
-    <row r="22" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="64" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" s="42">
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
+      <c r="V21" s="27"/>
+      <c r="W21" s="27"/>
+      <c r="X21" s="28"/>
+    </row>
+    <row r="22" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="14">
         <f>+'[1]S-2'!B21</f>
         <v>526</v>
       </c>
-      <c r="C22" s="65">
+      <c r="C22" s="31">
         <f>'[1]S-2'!D21</f>
         <v>587</v>
       </c>
-      <c r="D22" s="44">
+      <c r="D22" s="16">
         <f>'[1]S-2'!F21</f>
         <v>485</v>
       </c>
-      <c r="E22" s="43">
+      <c r="E22" s="15">
         <f>+G22+F22</f>
         <v>460</v>
       </c>
-      <c r="F22" s="45">
+      <c r="F22" s="17">
         <f>+'[1]S-3'!C22</f>
         <v>115</v>
       </c>
-      <c r="G22" s="45">
+      <c r="G22" s="17">
         <f>+'[1]S-3'!D22</f>
         <v>345</v>
       </c>
-      <c r="H22" s="47">
+      <c r="H22" s="19">
         <f>'[1]S-4'!B21</f>
         <v>395</v>
       </c>
-      <c r="I22" s="66">
+      <c r="I22" s="32">
         <f>'[1]S-4'!L21</f>
         <v>53.5</v>
       </c>
-      <c r="J22" s="67">
+      <c r="J22" s="33">
         <f>+'[1]S-9'!I20</f>
         <v>57</v>
       </c>
-      <c r="K22" s="68">
+      <c r="K22" s="34">
         <f>+'[1]S-9'!M20</f>
         <v>86.5</v>
       </c>
-      <c r="L22" s="68">
+      <c r="L22" s="34">
         <f>+J22+K22</f>
         <v>143.5</v>
       </c>
-      <c r="M22" s="46">
+      <c r="M22" s="18">
         <f>'[1]S-9'!N20</f>
         <v>423</v>
       </c>
-      <c r="N22" s="69">
+      <c r="N22" s="35">
         <f>'[1]S-2'!I21</f>
         <v>5.71</v>
       </c>
-      <c r="O22" s="48">
+      <c r="O22" s="35">
         <v>42.5</v>
       </c>
-      <c r="P22" s="49">
+      <c r="P22" s="35">
         <v>184</v>
       </c>
-      <c r="Q22" s="50">
+      <c r="Q22" s="35">
         <v>40</v>
       </c>
-      <c r="R22" s="51">
+      <c r="R22" s="35">
         <v>13.5</v>
       </c>
     </row>
-    <row r="23" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="64" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="52">
+    <row r="23" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="20">
         <f>+'[1]S-2'!B22</f>
         <v>526</v>
       </c>
-      <c r="C23" s="70">
+      <c r="C23" s="36">
         <f>'[1]S-2'!D22</f>
         <v>526</v>
       </c>
-      <c r="D23" s="44">
+      <c r="D23" s="16">
         <f>'[1]S-2'!F22</f>
         <v>434</v>
       </c>
-      <c r="E23" s="47">
+      <c r="E23" s="19">
         <f>+G23+F23</f>
         <v>417</v>
       </c>
-      <c r="F23" s="46">
+      <c r="F23" s="18">
         <f>+'[1]S-3'!C23</f>
         <v>109</v>
       </c>
-      <c r="G23" s="46">
+      <c r="G23" s="18">
         <f>+'[1]S-3'!D23</f>
         <v>308</v>
       </c>
-      <c r="H23" s="47">
+      <c r="H23" s="19">
         <f>'[1]S-4'!B22</f>
         <v>365</v>
       </c>
-      <c r="I23" s="66">
+      <c r="I23" s="32">
         <f>'[1]S-4'!L22</f>
         <v>49</v>
       </c>
-      <c r="J23" s="71">
+      <c r="J23" s="37">
         <f>+'[1]S-9'!I21</f>
         <v>51</v>
       </c>
-      <c r="K23" s="68">
+      <c r="K23" s="34">
         <f>+'[1]S-9'!M21</f>
         <v>77.5</v>
       </c>
-      <c r="L23" s="68">
+      <c r="L23" s="34">
         <f>+J23+K23</f>
         <v>128.5</v>
       </c>
-      <c r="M23" s="46">
+      <c r="M23" s="18">
         <f>'[1]S-9'!N21</f>
         <v>389</v>
       </c>
-      <c r="N23" s="69">
+      <c r="N23" s="35">
         <f>'[1]S-2'!I22</f>
         <v>0.34</v>
       </c>
-      <c r="O23" s="48">
+      <c r="O23" s="35">
         <v>36.5</v>
       </c>
-      <c r="P23" s="49">
+      <c r="P23" s="35">
         <v>175</v>
       </c>
-      <c r="Q23" s="50">
+      <c r="Q23" s="35">
         <v>38</v>
       </c>
-      <c r="R23" s="49">
+      <c r="R23" s="35">
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:24" s="20" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="64" t="s">
-        <v>38</v>
-      </c>
-      <c r="B24" s="52">
+    <row r="24" spans="1:24" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="20">
         <f>+'[1]S-2'!B23</f>
         <v>526</v>
       </c>
-      <c r="C24" s="72">
+      <c r="C24" s="38">
         <f>'[1]S-2'!D23</f>
         <v>587</v>
       </c>
-      <c r="D24" s="53">
+      <c r="D24" s="21">
         <f>'[1]S-2'!F23</f>
         <v>485</v>
       </c>
-      <c r="E24" s="53">
+      <c r="E24" s="21">
         <f>+G24+F24</f>
         <v>466</v>
       </c>
-      <c r="F24" s="46">
+      <c r="F24" s="18">
         <f>+'[1]S-3'!C24</f>
         <v>121</v>
       </c>
-      <c r="G24" s="46">
+      <c r="G24" s="18">
         <f>+'[1]S-3'!D24</f>
         <v>345</v>
       </c>
-      <c r="H24" s="47">
+      <c r="H24" s="19">
         <f>'[1]S-4'!B23</f>
         <v>405</v>
       </c>
-      <c r="I24" s="66">
+      <c r="I24" s="32">
         <f>'[1]S-4'!L23</f>
         <v>53.5</v>
       </c>
-      <c r="J24" s="71">
+      <c r="J24" s="37">
         <f>+'[1]S-9'!I22</f>
         <v>57</v>
       </c>
-      <c r="K24" s="68">
+      <c r="K24" s="34">
         <f>+'[1]S-9'!M22</f>
         <v>86.5</v>
       </c>
-      <c r="L24" s="68">
+      <c r="L24" s="34">
         <f>+J24+K24</f>
         <v>143.5</v>
       </c>
-      <c r="M24" s="46">
+      <c r="M24" s="18">
         <f>'[1]S-9'!N22</f>
         <v>433</v>
       </c>
-      <c r="N24" s="69">
+      <c r="N24" s="35">
         <f>'[1]S-2'!I23</f>
         <v>0.42</v>
       </c>
-      <c r="O24" s="48">
+      <c r="O24" s="35">
         <v>42.5</v>
       </c>
-      <c r="P24" s="49">
+      <c r="P24" s="35">
         <v>194</v>
       </c>
-      <c r="Q24" s="50">
+      <c r="Q24" s="35">
         <v>40</v>
       </c>
-      <c r="R24" s="54">
+      <c r="R24" s="35">
         <v>13.5</v>
       </c>
     </row>
-    <row r="25" spans="1:24" s="63" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="55" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25" s="73">
+    <row r="25" spans="1:24" s="29" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="39">
         <f>(B22*31+B23*28+B24*31)/90</f>
         <v>526</v>
       </c>
-      <c r="C25" s="57">
+      <c r="C25" s="24">
         <f t="shared" ref="C25:N25" si="3">SUM(C22:C24)</f>
         <v>1700</v>
       </c>
-      <c r="D25" s="57">
+      <c r="D25" s="24">
         <f t="shared" si="3"/>
         <v>1404</v>
       </c>
-      <c r="E25" s="57">
+      <c r="E25" s="24">
         <f t="shared" si="3"/>
         <v>1343</v>
       </c>
-      <c r="F25" s="57">
+      <c r="F25" s="24">
         <f>SUM(F22:F24)</f>
         <v>345</v>
       </c>
-      <c r="G25" s="57">
+      <c r="G25" s="24">
         <f t="shared" si="3"/>
         <v>998</v>
       </c>
-      <c r="H25" s="57">
+      <c r="H25" s="24">
         <f t="shared" si="3"/>
         <v>1165</v>
       </c>
-      <c r="I25" s="58">
+      <c r="I25" s="25">
         <f t="shared" si="3"/>
         <v>156</v>
       </c>
-      <c r="J25" s="58">
+      <c r="J25" s="25">
         <f t="shared" si="3"/>
         <v>165</v>
       </c>
-      <c r="K25" s="58">
+      <c r="K25" s="25">
         <f t="shared" si="3"/>
         <v>250.5</v>
       </c>
-      <c r="L25" s="58">
+      <c r="L25" s="25">
         <f t="shared" si="3"/>
         <v>415.5</v>
       </c>
-      <c r="M25" s="56">
+      <c r="M25" s="23">
         <f t="shared" si="3"/>
         <v>1245</v>
       </c>
-      <c r="N25" s="59">
+      <c r="N25" s="26">
         <f t="shared" si="3"/>
         <v>6.47</v>
       </c>
-      <c r="O25" s="48">
+      <c r="O25" s="26">
         <v>121.5</v>
       </c>
-      <c r="P25" s="60">
+      <c r="P25" s="26">
         <v>553</v>
       </c>
-      <c r="Q25" s="60">
+      <c r="Q25" s="26">
         <v>118</v>
       </c>
-      <c r="R25" s="60">
+      <c r="R25" s="26">
         <v>38</v>
       </c>
-      <c r="S25" s="61"/>
-      <c r="T25" s="61"/>
-      <c r="U25" s="61"/>
-      <c r="V25" s="61"/>
-      <c r="W25" s="61"/>
-      <c r="X25" s="62"/>
-    </row>
-    <row r="26" spans="1:24" s="78" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="74" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" s="75">
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
+      <c r="V25" s="27"/>
+      <c r="W25" s="27"/>
+      <c r="X25" s="28"/>
+    </row>
+    <row r="26" spans="1:24" s="41" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" s="65">
         <f>(B13*91+B17*92+B21*92+B25*90)/365</f>
         <v>524.9780821917808</v>
       </c>
-      <c r="C26" s="75">
+      <c r="C26" s="65">
         <f>SUM(C13,C17,C21,C25)</f>
         <v>6530</v>
       </c>
-      <c r="D26" s="75">
+      <c r="D26" s="65">
         <f t="shared" ref="D26:N26" si="4">SUM(D13,D17,D21,D25)</f>
         <v>5500</v>
       </c>
-      <c r="E26" s="75">
+      <c r="E26" s="65">
         <f t="shared" si="4"/>
         <v>5250</v>
       </c>
-      <c r="F26" s="75">
+      <c r="F26" s="65">
         <f>SUM(F13,F17,F21,F25)</f>
         <v>1350</v>
       </c>
-      <c r="G26" s="75">
+      <c r="G26" s="65">
         <f t="shared" si="4"/>
         <v>3900</v>
       </c>
-      <c r="H26" s="75">
+      <c r="H26" s="65">
         <f t="shared" si="4"/>
         <v>4576</v>
       </c>
-      <c r="I26" s="75">
+      <c r="I26" s="65">
         <f t="shared" si="4"/>
         <v>610</v>
       </c>
-      <c r="J26" s="75">
+      <c r="J26" s="65">
         <f t="shared" si="4"/>
         <v>660</v>
       </c>
-      <c r="K26" s="75">
+      <c r="K26" s="65">
         <f>SUM(K13,K17,K21,K25)</f>
         <v>1000</v>
       </c>
-      <c r="L26" s="75">
+      <c r="L26" s="65">
         <f>SUM(L13,L17,L21,L25)</f>
         <v>1660</v>
       </c>
-      <c r="M26" s="75">
+      <c r="M26" s="65">
         <f t="shared" si="4"/>
         <v>4921</v>
       </c>
-      <c r="N26" s="76">
+      <c r="N26" s="60">
         <f t="shared" si="4"/>
         <v>35.11</v>
       </c>
-      <c r="O26" s="48">
+      <c r="O26" s="60">
         <v>508</v>
       </c>
-      <c r="P26" s="77">
+      <c r="P26" s="60">
         <f>SUM(P13,P17,P21,P25)</f>
         <v>2143</v>
       </c>
-      <c r="Q26" s="77">
+      <c r="Q26" s="60">
         <f t="shared" ref="Q26:R26" si="5">SUM(Q13,Q17,Q21,Q25)</f>
         <v>467</v>
       </c>
-      <c r="R26" s="77">
+      <c r="R26" s="60">
         <f t="shared" si="5"/>
         <v>143</v>
       </c>
     </row>
-    <row r="27" spans="1:24" s="78" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="79" t="s">
+    <row r="27" spans="1:24" s="41" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="67"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="66"/>
+      <c r="H27" s="66"/>
+      <c r="I27" s="67"/>
+      <c r="J27" s="67"/>
+      <c r="K27" s="67"/>
+      <c r="L27" s="67"/>
+      <c r="M27" s="67"/>
+      <c r="N27" s="61"/>
+      <c r="O27" s="61"/>
+      <c r="P27" s="61"/>
+      <c r="Q27" s="61"/>
+      <c r="R27" s="61"/>
+      <c r="S27" s="43"/>
+      <c r="T27" s="43"/>
+      <c r="U27" s="43"/>
+      <c r="V27" s="43"/>
+      <c r="W27" s="43"/>
+      <c r="X27" s="44"/>
+    </row>
+    <row r="28" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="45"/>
+      <c r="B28" s="45"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="47"/>
+      <c r="L28" s="47"/>
+      <c r="M28" s="48"/>
+    </row>
+    <row r="29" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="49"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="49"/>
+      <c r="K29" s="49"/>
+      <c r="L29" s="49"/>
+      <c r="M29" s="49"/>
+    </row>
+    <row r="30" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="49"/>
+      <c r="G30" s="49"/>
+      <c r="H30" s="49"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="49"/>
+      <c r="K30" s="49"/>
+      <c r="L30" s="49"/>
+      <c r="M30" s="49"/>
+      <c r="N30" s="49"/>
+    </row>
+    <row r="31" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="51"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="63"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+    </row>
+    <row r="33" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="80"/>
-      <c r="C27" s="81"/>
-      <c r="D27" s="81"/>
-      <c r="E27" s="81"/>
-      <c r="F27" s="81"/>
-      <c r="G27" s="81"/>
-      <c r="H27" s="81"/>
-      <c r="I27" s="80"/>
-      <c r="J27" s="80"/>
-      <c r="K27" s="80"/>
-      <c r="L27" s="80"/>
-      <c r="M27" s="80"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="48"/>
-      <c r="P27" s="83"/>
-      <c r="Q27" s="83"/>
-      <c r="R27" s="83"/>
-      <c r="S27" s="84"/>
-      <c r="T27" s="84"/>
-      <c r="U27" s="84"/>
-      <c r="V27" s="84"/>
-      <c r="W27" s="84"/>
-      <c r="X27" s="85"/>
-    </row>
-    <row r="28" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="86"/>
-      <c r="B28" s="86"/>
-      <c r="C28" s="86"/>
-      <c r="D28" s="87"/>
-      <c r="E28" s="88"/>
-      <c r="F28" s="88"/>
-      <c r="G28" s="88"/>
-      <c r="H28" s="88"/>
-      <c r="I28" s="88"/>
-      <c r="J28" s="88"/>
-      <c r="K28" s="88"/>
-      <c r="L28" s="88"/>
-      <c r="M28" s="89"/>
-    </row>
-    <row r="29" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="90"/>
-      <c r="D29" s="90"/>
-      <c r="E29" s="90"/>
-      <c r="F29" s="90"/>
-      <c r="G29" s="90"/>
-      <c r="H29" s="90"/>
-      <c r="I29" s="90"/>
-      <c r="J29" s="90"/>
-      <c r="K29" s="90"/>
-      <c r="L29" s="90"/>
-      <c r="M29" s="90"/>
-    </row>
-    <row r="30" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="7"/>
-      <c r="B30" s="91"/>
-      <c r="C30" s="90"/>
-      <c r="D30" s="90"/>
-      <c r="E30" s="90"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="90"/>
-      <c r="H30" s="90"/>
-      <c r="I30" s="90"/>
-      <c r="J30" s="90"/>
-      <c r="K30" s="90"/>
-      <c r="L30" s="90"/>
-      <c r="M30" s="90"/>
-      <c r="N30" s="90"/>
-    </row>
-    <row r="31" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="92"/>
-      <c r="E31" s="93"/>
-      <c r="F31" s="94"/>
-      <c r="G31" s="95"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-    </row>
-    <row r="33" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="96" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" s="96"/>
-      <c r="C33" s="96"/>
-      <c r="D33" s="96"/>
-      <c r="E33" s="96"/>
-      <c r="F33" s="96"/>
-      <c r="G33" s="96"/>
-      <c r="H33" s="96"/>
-      <c r="I33" s="96"/>
-      <c r="J33" s="96"/>
-      <c r="K33" s="96"/>
-      <c r="L33" s="96"/>
-      <c r="M33" s="96"/>
-      <c r="N33" s="96"/>
+      <c r="B33" s="64"/>
+      <c r="C33" s="64"/>
+      <c r="D33" s="64"/>
+      <c r="E33" s="64"/>
+      <c r="F33" s="64"/>
+      <c r="G33" s="64"/>
+      <c r="H33" s="64"/>
+      <c r="I33" s="64"/>
+      <c r="J33" s="64"/>
+      <c r="K33" s="64"/>
+      <c r="L33" s="64"/>
+      <c r="M33" s="64"/>
+      <c r="N33" s="64"/>
     </row>
     <row r="37" spans="1:14" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="B37" s="97"/>
-      <c r="C37" s="98"/>
-      <c r="D37" s="98"/>
-      <c r="E37" s="99"/>
-      <c r="F37" s="98"/>
-      <c r="G37" s="98"/>
-      <c r="H37" s="98"/>
-      <c r="I37" s="98"/>
-      <c r="J37" s="98"/>
-      <c r="K37" s="98"/>
-      <c r="L37" s="99"/>
-      <c r="M37" s="98"/>
-      <c r="N37" s="100"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="54"/>
+      <c r="D37" s="54"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
+      <c r="H37" s="54"/>
+      <c r="I37" s="54"/>
+      <c r="J37" s="54"/>
+      <c r="K37" s="54"/>
+      <c r="L37" s="55"/>
+      <c r="M37" s="54"/>
+      <c r="N37" s="56"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="B38" s="101"/>
-      <c r="C38" s="101"/>
-      <c r="D38" s="101"/>
-      <c r="E38" s="101"/>
-      <c r="F38" s="101"/>
-      <c r="G38" s="101"/>
-      <c r="H38" s="101"/>
-      <c r="I38" s="101"/>
-      <c r="J38" s="101"/>
-      <c r="K38" s="101"/>
-      <c r="L38" s="101"/>
-      <c r="M38" s="101"/>
-      <c r="N38" s="101"/>
+      <c r="B38" s="57"/>
+      <c r="C38" s="57"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="57"/>
+      <c r="F38" s="57"/>
+      <c r="G38" s="57"/>
+      <c r="H38" s="57"/>
+      <c r="I38" s="57"/>
+      <c r="J38" s="57"/>
+      <c r="K38" s="57"/>
+      <c r="L38" s="57"/>
+      <c r="M38" s="57"/>
+      <c r="N38" s="57"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="B39" s="102"/>
-      <c r="C39" s="102"/>
-      <c r="D39" s="102"/>
-      <c r="E39" s="102"/>
-      <c r="F39" s="102"/>
-      <c r="G39" s="102"/>
-      <c r="H39" s="102"/>
-      <c r="I39" s="102"/>
-      <c r="J39" s="102"/>
-      <c r="K39" s="102"/>
-      <c r="L39" s="102"/>
-      <c r="M39" s="102"/>
-      <c r="N39" s="102"/>
+      <c r="B39" s="58"/>
+      <c r="C39" s="58"/>
+      <c r="D39" s="58"/>
+      <c r="E39" s="58"/>
+      <c r="F39" s="58"/>
+      <c r="G39" s="58"/>
+      <c r="H39" s="58"/>
+      <c r="I39" s="58"/>
+      <c r="J39" s="58"/>
+      <c r="K39" s="58"/>
+      <c r="L39" s="58"/>
+      <c r="M39" s="58"/>
+      <c r="N39" s="58"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="B40" s="102"/>
-      <c r="C40" s="102"/>
-      <c r="D40" s="102"/>
-      <c r="E40" s="102"/>
-      <c r="F40" s="102"/>
-      <c r="G40" s="102"/>
-      <c r="H40" s="102"/>
-      <c r="I40" s="102"/>
-      <c r="J40" s="102"/>
-      <c r="K40" s="102"/>
-      <c r="L40" s="102"/>
-      <c r="M40" s="102"/>
-      <c r="N40" s="102"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="58"/>
+      <c r="H40" s="58"/>
+      <c r="I40" s="58"/>
+      <c r="J40" s="58"/>
+      <c r="K40" s="58"/>
+      <c r="L40" s="58"/>
+      <c r="M40" s="58"/>
+      <c r="N40" s="58"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="B41" s="102"/>
-      <c r="C41" s="102"/>
-      <c r="D41" s="102"/>
-      <c r="E41" s="102"/>
-      <c r="F41" s="102"/>
-      <c r="G41" s="102"/>
-      <c r="H41" s="102"/>
-      <c r="I41" s="102"/>
-      <c r="J41" s="102"/>
-      <c r="K41" s="102"/>
-      <c r="L41" s="102"/>
-      <c r="M41" s="102"/>
-      <c r="N41" s="102"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="58"/>
+      <c r="G41" s="58"/>
+      <c r="H41" s="58"/>
+      <c r="I41" s="58"/>
+      <c r="J41" s="58"/>
+      <c r="K41" s="58"/>
+      <c r="L41" s="58"/>
+      <c r="M41" s="58"/>
+      <c r="N41" s="58"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="B42" s="102"/>
-      <c r="C42" s="102"/>
-      <c r="D42" s="102"/>
-      <c r="E42" s="102"/>
-      <c r="F42" s="102"/>
-      <c r="G42" s="102"/>
-      <c r="H42" s="102"/>
-      <c r="I42" s="102"/>
-      <c r="J42" s="102"/>
-      <c r="K42" s="102"/>
-      <c r="L42" s="102"/>
-      <c r="M42" s="102"/>
-      <c r="N42" s="102"/>
+      <c r="B42" s="58"/>
+      <c r="C42" s="58"/>
+      <c r="D42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="58"/>
+      <c r="G42" s="58"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
+      <c r="J42" s="58"/>
+      <c r="K42" s="58"/>
+      <c r="L42" s="58"/>
+      <c r="M42" s="58"/>
+      <c r="N42" s="58"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="C43" s="103"/>
-      <c r="D43" s="103"/>
-      <c r="E43" s="103"/>
-      <c r="F43" s="103"/>
-      <c r="G43" s="103"/>
-      <c r="H43" s="103"/>
-      <c r="I43" s="103"/>
-      <c r="J43" s="103"/>
-      <c r="K43" s="103"/>
-      <c r="L43" s="103"/>
-      <c r="M43" s="103"/>
-      <c r="N43" s="103"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
+      <c r="H43" s="59"/>
+      <c r="I43" s="59"/>
+      <c r="J43" s="59"/>
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
+      <c r="M43" s="59"/>
+      <c r="N43" s="59"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="C44" s="103"/>
-      <c r="D44" s="103"/>
-      <c r="E44" s="103"/>
-      <c r="F44" s="103"/>
-      <c r="G44" s="103"/>
-      <c r="H44" s="103"/>
-      <c r="I44" s="103"/>
-      <c r="J44" s="103"/>
-      <c r="K44" s="103"/>
-      <c r="L44" s="103"/>
-      <c r="M44" s="103"/>
-      <c r="N44" s="103"/>
+      <c r="C44" s="59"/>
+      <c r="D44" s="59"/>
+      <c r="E44" s="59"/>
+      <c r="F44" s="59"/>
+      <c r="G44" s="59"/>
+      <c r="H44" s="59"/>
+      <c r="I44" s="59"/>
+      <c r="J44" s="59"/>
+      <c r="K44" s="59"/>
+      <c r="L44" s="59"/>
+      <c r="M44" s="59"/>
+      <c r="N44" s="59"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="C45" s="103"/>
-      <c r="D45" s="103"/>
-      <c r="E45" s="103"/>
-      <c r="F45" s="103"/>
-      <c r="G45" s="103"/>
-      <c r="H45" s="103"/>
-      <c r="I45" s="103"/>
-      <c r="J45" s="103"/>
-      <c r="K45" s="103"/>
-      <c r="L45" s="103"/>
-      <c r="M45" s="103"/>
-      <c r="N45" s="103"/>
+      <c r="C45" s="59"/>
+      <c r="D45" s="59"/>
+      <c r="E45" s="59"/>
+      <c r="F45" s="59"/>
+      <c r="G45" s="59"/>
+      <c r="H45" s="59"/>
+      <c r="I45" s="59"/>
+      <c r="J45" s="59"/>
+      <c r="K45" s="59"/>
+      <c r="L45" s="59"/>
+      <c r="M45" s="59"/>
+      <c r="N45" s="59"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="C46" s="103"/>
-      <c r="D46" s="103"/>
-      <c r="E46" s="103"/>
-      <c r="F46" s="103"/>
-      <c r="G46" s="103"/>
-      <c r="H46" s="103"/>
-      <c r="I46" s="103"/>
-      <c r="J46" s="103"/>
-      <c r="K46" s="103"/>
-      <c r="L46" s="103"/>
-      <c r="M46" s="103"/>
-      <c r="N46" s="103"/>
+      <c r="C46" s="59"/>
+      <c r="D46" s="59"/>
+      <c r="E46" s="59"/>
+      <c r="F46" s="59"/>
+      <c r="G46" s="59"/>
+      <c r="H46" s="59"/>
+      <c r="I46" s="59"/>
+      <c r="J46" s="59"/>
+      <c r="K46" s="59"/>
+      <c r="L46" s="59"/>
+      <c r="M46" s="59"/>
+      <c r="N46" s="59"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="C47" s="102"/>
-      <c r="D47" s="102"/>
-      <c r="E47" s="102"/>
-      <c r="F47" s="102"/>
-      <c r="G47" s="102"/>
-      <c r="H47" s="102"/>
-      <c r="I47" s="102"/>
-      <c r="J47" s="102"/>
-      <c r="K47" s="102"/>
-      <c r="L47" s="102"/>
-      <c r="M47" s="102"/>
-      <c r="N47" s="102"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="58"/>
+      <c r="E47" s="58"/>
+      <c r="F47" s="58"/>
+      <c r="G47" s="58"/>
+      <c r="H47" s="58"/>
+      <c r="I47" s="58"/>
+      <c r="J47" s="58"/>
+      <c r="K47" s="58"/>
+      <c r="L47" s="58"/>
+      <c r="M47" s="58"/>
+      <c r="N47" s="58"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="N26:N27"/>
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="Q26:Q27"/>
-    <mergeCell ref="R26:R27"/>
-    <mergeCell ref="F31:G31"/>
+  <mergeCells count="39">
+    <mergeCell ref="O6:O9"/>
+    <mergeCell ref="P6:P9"/>
+    <mergeCell ref="Q6:Q9"/>
+    <mergeCell ref="R6:R9"/>
+    <mergeCell ref="O26:O27"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="I6:I9"/>
+    <mergeCell ref="J6:L7"/>
+    <mergeCell ref="M6:M9"/>
+    <mergeCell ref="N6:N9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
     <mergeCell ref="A33:N33"/>
     <mergeCell ref="H26:H27"/>
     <mergeCell ref="I26:I27"/>
@@ -3383,26 +3356,15 @@
     <mergeCell ref="E26:E27"/>
     <mergeCell ref="F26:F27"/>
     <mergeCell ref="G26:G27"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="I6:I9"/>
-    <mergeCell ref="J6:L7"/>
-    <mergeCell ref="M6:M9"/>
-    <mergeCell ref="N6:N9"/>
+    <mergeCell ref="N26:N27"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="Q26:Q27"/>
+    <mergeCell ref="R26:R27"/>
+    <mergeCell ref="F31:G31"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0" right="0" top="0.5" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0.17" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="86" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>